<commit_message>
chore: sync DramaTV community project state
</commit_message>
<xml_diff>
--- a/docs/03_架构/DramaTV社区功能规划清单-已同步.xlsx
+++ b/docs/03_架构/DramaTV社区功能规划清单-已同步.xlsx
@@ -570,8 +570,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J109"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:J115"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -780,12 +780,12 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Markdown 帖子</t>
+          <t>图文帖子 / 富文本帖子</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>独立讨论内容，可插图片/视频附件，但附件不改变帖子主类型</t>
+          <t>独立讨论内容，可插图片/视频附件；帖子正文已升级为富文本编辑与渲染，附件不改变帖子主类型</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -1045,7 +1045,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>展示提示词、视频、图片、工作流等 PGC 内容池；筛选项已按图片/短篇/工作流方向收口</t>
+          <t>展示提示词、工作流等 PGC 内容池；已支持按全部/工作流/视频提示词/图片提示词切换，并开始承接模型/题材分类治理</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -1125,12 +1125,12 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>视频 Prompt / 图片 Prompt / 工作流占位发布统一走 /publish；讨论帖子独立走 /discussions/new，两个发布入口已分离</t>
+          <t>视频 Prompt / 图片 Prompt / 工作流占位统一走 /publish；表单会随类型切换上传区、提示词区与分类标签，讨论帖子独立走 /discussions/new</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>开发中</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1140,12 +1140,12 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>V1.1 产品补强</t>
+          <t>V1.1 内容发布</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -1329,7 +1329,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Markdown 正文阅读、帖子互动、评论区；页面随帖子长度自然撑开</t>
+          <t>富文本正文阅读、帖子互动、评论区；页面随帖子长度自然撑开</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1349,7 +1349,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -1717,12 +1717,12 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>前台已按游客和登录用户区分；创作者能力继续跟发布链路绑定</t>
+          <t>前台已按游客 / 登录用户收口；创作者通过真实发布、/me 个人中心、通知与互动能力形成可用闭环</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
-          <t>开发中</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="H27" s="8" t="inlineStr">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>后台角色已收口为 admin/operator/moderator 三类，独立后台 apps/admin 已按这套边界推进</t>
+          <t>后台角色已收口为 admin/operator/moderator 三类，独立后台 apps/admin 已按这套边界推进并接入主要治理接口；更细 RBAC 矩阵待补</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
@@ -1777,7 +1777,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -2057,7 +2057,7 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>独立帖子内容，不再在用户端暴露历史绑定对象 UI</t>
+          <t>独立帖子内容，正文支持富文本存储/渲染，不再在用户端暴露历史绑定对象 UI</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -2277,7 +2277,7 @@
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>当前本地仍支持本地上传；云测试已接通后端写 OSS，前端 100MB、后端策略 300MB；后续改预签名直传与分片上传</t>
+          <t>当前本地支持本地上传，云测试已接通后端写私有 OSS；前端 100MB、后端 300MB，并已补封面/preview 派生、去重与代理展示，后续改预签名直传与分片上传</t>
         </is>
       </c>
       <c r="G40" s="11" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Markdown 编辑</t>
+          <t>富文本编辑器</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
@@ -2401,7 +2401,7 @@
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>独立帖子发布页已落地，支持 Markdown 正文、图片/视频插入与发布；已按现有社区风格完成一轮精修</t>
+          <t>独立帖子发布页已升级为 TipTap 富文本编辑器，支持标题/字号/颜色/图片/视频插入与发布，并已按社区风格完成一轮精修</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -2421,7 +2421,7 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -2701,7 +2701,7 @@
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>详情页评论、楼中楼、评论点赞已跑通本地链路；评论开关与作者删评第一版已完成</t>
+          <t>详情页评论、两层楼中楼、就地回复、折叠展开、评论点赞已跑通；评论开关与作者删评第一版已完成</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -2877,12 +2877,12 @@
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>顶栏铃铛已支持最近点赞、收藏、评论、回复通知与未读红点；系统消息与审核消息后续补齐</t>
+          <t>顶栏铃铛已支持最近点赞、收藏、评论、回复通知、已读清红点与头像跳转；系统消息与审核消息后续补齐</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>开发中</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="H54" s="8" t="inlineStr">
@@ -2897,7 +2897,7 @@
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -3189,12 +3189,12 @@
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>审核后台已落地第一期：/api/admin/moderation 与 /admin/moderation 已接通真实列表、详情、通过、驳回、下线、恢复；更细审核规则待补</t>
+          <t>审核后台第一期已落地：/api/admin/moderation 与 /admin/moderation 已接通真实列表、详情、通过、驳回、下线、恢复；更细规则与批量操作待补</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>开发中</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="H61" s="8" t="inlineStr">
@@ -3209,7 +3209,7 @@
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -3233,12 +3233,12 @@
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>report_tickets 已落地真实前后台链路：前台可举报，后台 /admin/reports 可查看与处理；阈值预警与更细状态流转待补</t>
+          <t>report_tickets 已落地真实前后台链路：前台可举报，后台 /admin/reports 可查看、处理并联动内容处置；阈值预警与更细状态流转待补</t>
         </is>
       </c>
       <c r="G62" s="12" t="inlineStr">
         <is>
-          <t>开发中</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="H62" s="8" t="inlineStr">
@@ -3253,7 +3253,7 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>评论内容已接文本敏感词、广告联系方式/链接、频率限制、重复内容拦截；帖子/标题/简介/Prompt 文案与图片/视频机审待补</t>
+          <t>评论内容已接文本敏感词、广告联系方式/链接、频率限制、重复内容拦截；帖子全文、标题/简介/Prompt 文案与图片/视频机审待补</t>
         </is>
       </c>
       <c r="G63" s="5" t="inlineStr">
@@ -3297,7 +3297,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -3369,7 +3369,7 @@
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>独立后台前端工程 apps/admin 已建立并运行，本地端口 3206，云镜像预留 3207；已接 auth/users/comments/moderation/reports/taxonomy/feed-ops/home</t>
+          <t>独立后台前端工程 apps/admin 已建立并运行，本地端口 3206，测试云公网入口 8.141.20.130:3206；已接 auth/dashboard/users/moderation/reports/comments/taxonomy/feed-ops/media-tasks/audit-logs/resources</t>
         </is>
       </c>
       <c r="G65" s="11" t="inlineStr">
@@ -3389,7 +3389,7 @@
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -3413,12 +3413,12 @@
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>聚合待审核数量、待处理举报、失败媒体任务和基本运营指标</t>
+          <t>仪表盘概览已落地第一期：聚合待审核数量、待处理举报、失败媒体任务、资源与账号等运营指标</t>
         </is>
       </c>
       <c r="G66" s="11" t="inlineStr">
         <is>
-          <t>待开发</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="H66" s="5" t="inlineStr">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -3541,7 +3541,7 @@
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>已接通真实用户列表；新增/禁用账号、重置密码、查看发布情况与更完整后台角色治理待补</t>
+          <t>已接通真实用户列表与创建本地账号；禁用账号、重置密码、查看发布情况与更完整后台角色治理待补</t>
         </is>
       </c>
       <c r="G69" s="11" t="inlineStr">
@@ -3561,7 +3561,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -3585,12 +3585,12 @@
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>已接通真实审核中心：统一处理视频 Prompt、图片 Prompt、工作流占位内容和帖子，支持通过/驳回/下线/恢复</t>
+          <t>已接通真实审核中心：统一处理视频 Prompt、图片 Prompt、工作流占位内容、帖子与视频作品，支持通过/驳回/下线/恢复</t>
         </is>
       </c>
       <c r="G70" s="11" t="inlineStr">
         <is>
-          <t>开发中</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="H70" s="5" t="inlineStr">
@@ -3605,7 +3605,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -3629,12 +3629,12 @@
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>已接通举报中心：处理帖子、评论、Prompt 内容与工作流占位内容的举报工单，并支持联动内容处置</t>
+          <t>已接通举报中心：处理帖子、评论、Prompt 内容、工作流占位内容与视频作品的举报工单，并支持联动内容处置</t>
         </is>
       </c>
       <c r="G71" s="11" t="inlineStr">
         <is>
-          <t>开发中</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="H71" s="5" t="inlineStr">
@@ -3649,7 +3649,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -3658,27 +3658,27 @@
       <c r="B72" s="6" t="n"/>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>评论治理</t>
+          <t>资源治理</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>评论治理</t>
+          <t>内容资源库</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>/admin/comments</t>
+          <t>/admin/resources</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>已接通评论治理：删除评论、隐藏/恢复评论、楼中楼上下文查看与目标内容关闭评论区</t>
+          <t>已接通真实资源列表、详情、上下线/恢复与媒体预览；可统一查看提示词、视频作品、工作流与帖子资源，批量治理与更细筛选待补</t>
         </is>
       </c>
       <c r="G72" s="11" t="inlineStr">
         <is>
-          <t>开发中</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -3693,7 +3693,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -3702,27 +3702,27 @@
       <c r="B73" s="6" t="n"/>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>运营配置</t>
+          <t>评论治理</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>首页/精选/讨论区排序</t>
+          <t>评论治理</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>/admin/feed-ops/*</t>
+          <t>/admin/comments</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>/admin/feed-ops/home 已接通真实读写；featured / discussions 的运营排序与展示位配置仍待补齐</t>
+          <t>已接通评论治理：删除评论、隐藏/恢复评论、楼中楼上下文查看、关闭评论区与恢复评论区</t>
         </is>
       </c>
       <c r="G73" s="11" t="inlineStr">
         <is>
-          <t>开发中</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -3737,27 +3737,31 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="74" ht="32" customHeight="1">
       <c r="A74" s="6" t="n"/>
       <c r="B74" s="6" t="n"/>
-      <c r="C74" s="7" t="n"/>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>运营配置</t>
+        </is>
+      </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>标签/模型/频道管理</t>
+          <t>落地页/首页/精选/讨论区编排</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>/admin/taxonomy</t>
+          <t>/admin/feed-ops/*</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>/admin/taxonomy 已接通真实分类统计与治理配置读写；前台曝光消费与更细运营规则待补</t>
+          <t>单入口 + 四个页面 tab 已落地并接通真实读写；候选池异步分页与更多展示位规则继续补齐</t>
         </is>
       </c>
       <c r="G74" s="11" t="inlineStr">
@@ -3777,36 +3781,32 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="75" ht="32" customHeight="1">
       <c r="A75" s="6" t="n"/>
       <c r="B75" s="6" t="n"/>
-      <c r="C75" s="2" t="inlineStr">
-        <is>
-          <t>媒体治理</t>
-        </is>
-      </c>
+      <c r="C75" s="7" t="n"/>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>媒体任务中心</t>
+          <t>标签/模型/频道管理</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>/admin/media-tasks</t>
+          <t>/admin/taxonomy</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>媒体任务中心仍待开发；后续统一排查上传失败、转码失败、抽帧/preview 失败与 OSS 资源状态</t>
+          <t>已接通真实分类统计与治理配置读写；前台发布页与精选页已开始消费模型/题材分类，更多运营规则与批量治理待补</t>
         </is>
       </c>
       <c r="G75" s="11" t="inlineStr">
         <is>
-          <t>待开发</t>
+          <t>开发中</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -3821,36 +3821,36 @@
       </c>
       <c r="J75" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="76" ht="32" customHeight="1">
       <c r="A76" s="6" t="n"/>
-      <c r="B76" s="7" t="n"/>
+      <c r="B76" s="6" t="n"/>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>后台操作日志</t>
+          <t>媒体治理</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>后台操作日志</t>
+          <t>媒体任务中心</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>/admin/audit-logs</t>
+          <t>/admin/media-tasks</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>后台操作日志仍待开发；后续记录后台账号操作、审核处置、运营变更与敏感修改</t>
+          <t>媒体任务中心第一期已落地：支持真实列表、详情、失败原因、回写结果与重试入口；更细聚合分析与批量操作待补</t>
         </is>
       </c>
       <c r="G76" s="11" t="inlineStr">
         <is>
-          <t>待开发</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="H76" s="5" t="inlineStr">
@@ -3865,84 +3865,84 @@
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="77" ht="32" customHeight="1">
       <c r="A77" s="6" t="n"/>
-      <c r="B77" s="2" t="inlineStr">
-        <is>
-          <t>媒体与云化</t>
-        </is>
-      </c>
+      <c r="B77" s="7" t="n"/>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>本地媒体</t>
+          <t>后台操作日志</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>本地文件存储</t>
+          <t>后台操作日志</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>tmp/media</t>
+          <t>/admin/audit-logs</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>本地开发仍支持 tmp/media 存储；云测试已不再只依赖本地文件，媒体链路开始转向 OSS</t>
+          <t>后台操作日志第一期已落地：支持真实列表、详情、requestId/traceId、请求路径与结果查看；更细审计策略待补</t>
         </is>
       </c>
       <c r="G77" s="11" t="inlineStr">
         <is>
-          <t>本地可用</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="H77" s="5" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>V1.1 云化改造</t>
+          <t>V1.2 后台系统</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="78" ht="32" customHeight="1">
       <c r="A78" s="6" t="n"/>
-      <c r="B78" s="6" t="n"/>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>媒体与云化</t>
+        </is>
+      </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>PGC 内容池</t>
+          <t>本地媒体</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>YouMind 资产导入</t>
+          <t>本地文件存储</t>
         </is>
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>图片提示词/视频提示词/可播放视频</t>
+          <t>tmp/media</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>YouMind 研究资产已持续导入本地与云测试内容池；云端统一作者为 community，作为社区初始数据</t>
-        </is>
-      </c>
-      <c r="G78" s="4" t="inlineStr">
-        <is>
-          <t>已完成</t>
+          <t>本地开发仍支持 tmp/media 存储；云测试已不再只依赖本地文件，媒体链路开始转向 OSS</t>
+        </is>
+      </c>
+      <c r="G78" s="11" t="inlineStr">
+        <is>
+          <t>本地可用</t>
         </is>
       </c>
       <c r="H78" s="5" t="inlineStr">
@@ -3966,27 +3966,27 @@
       <c r="B79" s="6" t="n"/>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>对象存储</t>
+          <t>PGC 内容池</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>OSS/S3/MinIO</t>
+          <t>YouMind 资产导入</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>storage_provider/bucket/object_key</t>
+          <t>图片提示词/视频提示词/可播放视频</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>云测试已接通私有 OSS + /media 代理 + Range 读取；CDN 与前端直传仍待补</t>
-        </is>
-      </c>
-      <c r="G79" s="5" t="inlineStr">
-        <is>
-          <t>开发中</t>
+          <t>YouMind 研究资产已持续导入本地与云测试内容池；云端统一作者为 community，作为社区初始数据，并已开始按模型/题材分类治理</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>已完成</t>
         </is>
       </c>
       <c r="H79" s="5" t="inlineStr">
@@ -4001,7 +4001,7 @@
       </c>
       <c r="J79" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -4010,27 +4010,27 @@
       <c r="B80" s="6" t="n"/>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>CDN 分发</t>
+          <t>对象存储</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>CDN URL</t>
+          <t>OSS/S3/MinIO</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>cover/poster/preview/source</t>
+          <t>storage_provider/bucket/object_key</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>前台资源后续应统一走 CDN 或受控 URL；当前云测试仍以 /media 代理为主，不直接暴露内部存储细节</t>
+          <t>云测试已接通私有 OSS + /media 代理；浏览器展示继续走后端代理读取，不直接暴露内部桶，后续再补 CDN 与前端直传</t>
         </is>
       </c>
       <c r="G80" s="5" t="inlineStr">
         <is>
-          <t>待开发</t>
+          <t>开发中</t>
         </is>
       </c>
       <c r="H80" s="5" t="inlineStr">
@@ -4045,7 +4045,7 @@
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -4054,27 +4054,27 @@
       <c r="B81" s="6" t="n"/>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>媒体处理</t>
+          <t>媒体网关</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>FFmpeg/Worker</t>
+          <t>/media 代理</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>转码/封面抽帧/preview 生成</t>
+          <t>ETag/Last-Modified/304/Range</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>已打通 async_task_records 与内部 callback 写回；真实转码、封面抽帧、preview Worker 仍待接入</t>
+          <t>私有 OSS 展示继续走社区后端 /media/** 代理；已补协商缓存、206 Range 与角色化 Cache-Control，当前无公网 OSS/CDN 也可稳定展示</t>
         </is>
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>开发中</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="H81" s="5" t="inlineStr">
@@ -4089,41 +4089,37 @@
       </c>
       <c r="J81" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="82" ht="32" customHeight="1">
       <c r="A82" s="6" t="n"/>
       <c r="B82" s="6" t="n"/>
-      <c r="C82" s="2" t="inlineStr">
-        <is>
-          <t>安全扫描</t>
-        </is>
-      </c>
+      <c r="C82" s="2" t="n"/>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>媒体安全</t>
+          <t>派生资源补齐</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>文件类型/大小/内容安全</t>
+          <t>cover/poster/preview backfill</t>
         </is>
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>已具备文件大小、类型与基础校验；生产级媒体安全扫描与更细合规检测待补</t>
+          <t>视频 &gt;6MB 自动补 preview + cover，图片大图自动补轻量 cover；云测试历史 backlog 已回补至 0</t>
         </is>
       </c>
       <c r="G82" s="5" t="inlineStr">
         <is>
-          <t>开发中</t>
-        </is>
-      </c>
-      <c r="H82" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="H82" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
@@ -4133,41 +4129,37 @@
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="83" ht="32" customHeight="1">
       <c r="A83" s="6" t="n"/>
       <c r="B83" s="6" t="n"/>
-      <c r="C83" s="2" t="inlineStr">
-        <is>
-          <t>大文件上传</t>
-        </is>
-      </c>
+      <c r="C83" s="2" t="n"/>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>预签名直传</t>
+          <t>资源去重</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>OSS multipart / resumable</t>
+          <t>checksum + object_key reuse</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>当前云测试为后端写 OSS；前端预签名直传、分片上传、断点续传与上传状态查询待补</t>
+          <t>上传与导入链路已接入 SHA-256 去重；同角色同内容复用物理对象，保留独立 media_assets 记录</t>
         </is>
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>待开发</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="H83" s="5" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr">
@@ -4177,80 +4169,76 @@
       </c>
       <c r="J83" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="84" ht="32" customHeight="1">
       <c r="A84" s="6" t="n"/>
-      <c r="B84" s="7" t="n"/>
-      <c r="C84" s="7" t="n"/>
+      <c r="B84" s="6" t="n"/>
+      <c r="C84" s="2" t="n"/>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>后端限流与大小策略</t>
+          <t>代理保护与观测</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>100MB/300MB 策略生产化</t>
+          <t>MEDIA_PROXY_BUSY / slow logs</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>已具备 100MB 前端 / 300MB 后端策略、请求头预检与实际写入字节兜底；上线后仍需按角色与内容类型统一限额</t>
+          <t>媒体代理已补限并发、503 忙碌保护、慢请求/失败结构化日志，云端专项验证已通过</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr">
         <is>
-          <t>开发中</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="H84" s="5" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>V1.1 云化改造</t>
+          <t>V1.1 运维化</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="85" ht="32" customHeight="1">
       <c r="A85" s="6" t="n"/>
-      <c r="B85" s="2" t="inlineStr">
-        <is>
-          <t>性能与异步</t>
-        </is>
-      </c>
+      <c r="B85" s="6" t="n"/>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>并发性能</t>
+          <t>CDN 分发</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>列表与详情读优化</t>
+          <t>CDN URL</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>分页/缓存/索引/CDN</t>
+          <t>cover/poster/preview/source</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>首页、精选、讨论页已完成一轮缓存、分页与列表读优化；压测、热点缓存策略和 CDN 命中优化待补</t>
+          <t>前台资源后续应统一走 CDN 或受控 URL；当前云测试仍以 /media 代理为主，不直接暴露内部存储细节</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>开发中</t>
+          <t>待开发</t>
         </is>
       </c>
       <c r="H85" s="5" t="inlineStr">
@@ -4260,7 +4248,7 @@
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>V1.1 生产化</t>
+          <t>V1.1 云化改造</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr">
@@ -4272,20 +4260,24 @@
     <row r="86" ht="32" customHeight="1">
       <c r="A86" s="6" t="n"/>
       <c r="B86" s="6" t="n"/>
-      <c r="C86" s="7" t="n"/>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>媒体处理</t>
+        </is>
+      </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>写接口保护</t>
+          <t>FFmpeg/Worker</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>限流/幂等/防重复提交</t>
+          <t>转码/封面抽帧/preview 生成</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>评论链路已补频率限制与重复内容拦截；发布、点赞、上传等全局限流与幂等体系待补</t>
+          <t>第一阶段媒体处理已可生成视频 preview/cover 与图片轻量 cover，并已打通历史 backfill；独立 Python Worker / 正式队列待接入</t>
         </is>
       </c>
       <c r="G86" s="5" t="inlineStr">
@@ -4293,19 +4285,19 @@
           <t>开发中</t>
         </is>
       </c>
-      <c r="H86" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="H86" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>V1.1 生产化</t>
+          <t>V1.1 云化改造</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -4314,22 +4306,22 @@
       <c r="B87" s="6" t="n"/>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>异步解耦</t>
+          <t>安全扫描</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>任务队列</t>
+          <t>媒体安全</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>Queue + Worker</t>
+          <t>文件类型/大小/内容安全</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>已具备 async_task_records 与 callback logs；正式队列、重试、死信和任务状态治理待补</t>
+          <t>已具备文件大小、类型与基础校验；生产级媒体安全扫描与更细合规检测待补</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">
@@ -4337,14 +4329,14 @@
           <t>开发中</t>
         </is>
       </c>
-      <c r="H87" s="5" t="inlineStr">
-        <is>
-          <t>P0</t>
+      <c r="H87" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>V1.1 生产化</t>
+          <t>V1.1 云化改造</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
@@ -4356,25 +4348,29 @@
     <row r="88" ht="32" customHeight="1">
       <c r="A88" s="6" t="n"/>
       <c r="B88" s="6" t="n"/>
-      <c r="C88" s="6" t="n"/>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>大文件上传</t>
+        </is>
+      </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>媒体处理任务</t>
+          <t>预签名直传</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>transcode / extract_cover / preview</t>
+          <t>OSS multipart / resumable</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>视频媒体任务已具备任务记录与回写位；真实 transcode / extract_cover / preview Worker 待接入</t>
+          <t>当前云测试为后端写 OSS；前端预签名直传、分片上传、断点续传与上传状态查询待补</t>
         </is>
       </c>
       <c r="G88" s="5" t="inlineStr">
         <is>
-          <t>开发中</t>
+          <t>待开发</t>
         </is>
       </c>
       <c r="H88" s="5" t="inlineStr">
@@ -4399,37 +4395,37 @@
       <c r="C89" s="7" t="n"/>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>画布复制任务</t>
+          <t>后端限流与大小策略</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>copy task / reconcile</t>
+          <t>100MB/300MB 策略生产化</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>当前已有 copy task 占位与 runtime 演示链路；真实画布复制、补偿、失败重试与进度回查待接入</t>
-        </is>
-      </c>
-      <c r="G89" s="12" t="inlineStr">
-        <is>
-          <t>已预留</t>
-        </is>
-      </c>
-      <c r="H89" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>已具备 100MB 前端 / 300MB 后端策略、请求头预检、实际写入字节兜底与大视频预处理阈值；上线后仍需按角色与内容类型统一限额</t>
+        </is>
+      </c>
+      <c r="G89" s="5" t="inlineStr">
+        <is>
+          <t>开发中</t>
+        </is>
+      </c>
+      <c r="H89" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>V1.1 画布对接</t>
+          <t>V1.1 云化改造</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -4437,27 +4433,27 @@
       <c r="A90" s="6" t="n"/>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>安全与风控</t>
+          <t>性能与异步</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>内容安全</t>
+          <t>并发性能</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>审核后台</t>
+          <t>列表与详情读优化</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>机审 + 人审 + 上下架</t>
+          <t>分页/缓存/索引/CDN</t>
         </is>
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>已完成评论实时拦截第一版；发布内容、媒体审核、后台人工处置与上下架闭环待补</t>
+          <t>首页、精选、讨论页已完成一轮分页/缓存/媒体分层读取优化；T6 已补悬浮播放回退、/media 协商缓存、Range 与代理保护，压测与 CDN 命中优化待补</t>
         </is>
       </c>
       <c r="G90" s="5" t="inlineStr">
@@ -4472,32 +4468,32 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>V1.2 后台系统</t>
+          <t>V1.1 生产化</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="91" ht="32" customHeight="1">
       <c r="A91" s="6" t="n"/>
       <c r="B91" s="6" t="n"/>
-      <c r="C91" s="6" t="n"/>
+      <c r="C91" s="7" t="n"/>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>评论/帖子风控</t>
+          <t>写接口保护</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>敏感词/广告/灌水/频率限制</t>
+          <t>限流/幂等/防重复提交</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>评论风控第一版已落地：敏感词、广告联系方式/URL、频率限制、重复文本拦截；帖子全文风控待补</t>
+          <t>评论链路已补频率限制与重复内容拦截；发布、点赞、上传等全局限流与幂等体系待补</t>
         </is>
       </c>
       <c r="G91" s="5" t="inlineStr">
@@ -4512,7 +4508,7 @@
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>V1.2 后台系统</t>
+          <t>V1.1 生产化</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr">
@@ -4524,20 +4520,24 @@
     <row r="92" ht="32" customHeight="1">
       <c r="A92" s="6" t="n"/>
       <c r="B92" s="6" t="n"/>
-      <c r="C92" s="7" t="n"/>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>异步解耦</t>
+        </is>
+      </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>上传安全</t>
+          <t>任务队列</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>mime 校验/病毒扫描/图片视频合规</t>
+          <t>Queue + Worker</t>
         </is>
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>已具备 mime/大小判断、请求头预检和实际写入字节兜底；病毒扫描、媒体合规与存储隔离策略待补</t>
+          <t>已具备 async_task_records、回调日志与 backfill 脚本；正式队列、独立 Worker、重试/死信与任务状态治理待补</t>
         </is>
       </c>
       <c r="G92" s="5" t="inlineStr">
@@ -4545,63 +4545,59 @@
           <t>开发中</t>
         </is>
       </c>
-      <c r="H92" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="H92" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>V1.1 云化改造</t>
+          <t>V1.1 生产化</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="93" ht="32" customHeight="1">
       <c r="A93" s="6" t="n"/>
       <c r="B93" s="6" t="n"/>
-      <c r="C93" s="2" t="inlineStr">
-        <is>
-          <t>账号防刷</t>
-        </is>
-      </c>
+      <c r="C93" s="6" t="n"/>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>机器注册防护</t>
+          <t>媒体处理任务</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>验证码/设备/IP/行为风控</t>
+          <t>transcode / extract_cover / preview</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>当前本地登录未做注册防刷；后续优先接公司画布登录，若自建注册则必须补风控</t>
+          <t>视频/图片媒体任务已具备任务记录、preview/cover 生成、历史 backfill 与回写位；更完整转码档位与独立 Worker 待补</t>
         </is>
       </c>
       <c r="G93" s="5" t="inlineStr">
         <is>
-          <t>待开发</t>
-        </is>
-      </c>
-      <c r="H93" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>开发中</t>
+        </is>
+      </c>
+      <c r="H93" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>V1.1 账号生产化</t>
+          <t>V1.1 云化改造</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -4611,22 +4607,22 @@
       <c r="C94" s="7" t="n"/>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>登录限流</t>
+          <t>画布复制任务</t>
         </is>
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>失败次数/IP/账号锁定</t>
+          <t>copy task / reconcile</t>
         </is>
       </c>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>登录接口上线前需限制暴力破解和撞库；当前本地登录只用于开发演示</t>
-        </is>
-      </c>
-      <c r="G94" s="5" t="inlineStr">
-        <is>
-          <t>待开发</t>
+          <t>当前已有 copy task 占位与 runtime 演示链路；真实画布复制、补偿、失败重试与进度回查待接入</t>
+        </is>
+      </c>
+      <c r="G94" s="12" t="inlineStr">
+        <is>
+          <t>已预留</t>
         </is>
       </c>
       <c r="H94" s="8" t="inlineStr">
@@ -4636,12 +4632,12 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>V1.1 账号生产化</t>
+          <t>V1.1 画布对接</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -4649,32 +4645,32 @@
       <c r="A95" s="6" t="n"/>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>推荐与运营</t>
+          <t>安全与风控</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>首页分发</t>
+          <t>内容安全</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>首页聚合</t>
+          <t>审核后台</t>
         </is>
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>/api/feed/home</t>
+          <t>机审 + 人审 + 上下架</t>
         </is>
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>首页和精选可从数据库读取内容，PGC 冷启动可演示</t>
-        </is>
-      </c>
-      <c r="G95" s="4" t="inlineStr">
-        <is>
-          <t>已完成</t>
+          <t>已完成评论实时拦截第一版，且前后台举报/审核/上下线链路已打通；发布内容机审、媒体审核与更细人工规则待补</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr">
+        <is>
+          <t>开发中</t>
         </is>
       </c>
       <c r="H95" s="5" t="inlineStr">
@@ -4684,39 +4680,35 @@
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>V1.0 本地闭环</t>
+          <t>V1.2 后台系统</t>
         </is>
       </c>
       <c r="J95" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="96" ht="32" customHeight="1">
       <c r="A96" s="6" t="n"/>
       <c r="B96" s="6" t="n"/>
-      <c r="C96" s="2" t="inlineStr">
-        <is>
-          <t>精选运营</t>
-        </is>
-      </c>
+      <c r="C96" s="6" t="n"/>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>运营精选</t>
+          <t>评论/帖子风控</t>
         </is>
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>featured/hot</t>
+          <t>敏感词/广告/灌水/频率限制</t>
         </is>
       </c>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>当前精选仍以业务查询和简单排序为主；后续由 /admin/feed-ops/featured 接管人工精选与排序</t>
-        </is>
-      </c>
-      <c r="G96" s="9" t="inlineStr">
+          <t>评论风控第一版已落地：敏感词、广告联系方式/URL、频率限制、重复文本拦截；帖子全文风控待补</t>
+        </is>
+      </c>
+      <c r="G96" s="5" t="inlineStr">
         <is>
           <t>开发中</t>
         </is>
@@ -4740,44 +4732,40 @@
     <row r="97" ht="32" customHeight="1">
       <c r="A97" s="6" t="n"/>
       <c r="B97" s="6" t="n"/>
-      <c r="C97" s="2" t="inlineStr">
-        <is>
-          <t>搜索能力</t>
-        </is>
-      </c>
+      <c r="C97" s="7" t="n"/>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>搜索引擎</t>
+          <t>上传安全</t>
         </is>
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>keyword/index</t>
+          <t>mime 校验/病毒扫描/图片视频合规</t>
         </is>
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>尚未接搜索引擎和索引更新任务，内容规模上来后再做</t>
+          <t>已具备 mime/大小判断、请求头预检和实际写入字节兜底；病毒扫描、媒体合规与存储隔离策略待补</t>
         </is>
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>待开发</t>
-        </is>
-      </c>
-      <c r="H97" s="11" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>开发中</t>
+        </is>
+      </c>
+      <c r="H97" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>V2.0 增强能力</t>
+          <t>V1.1 云化改造</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -4786,22 +4774,22 @@
       <c r="B98" s="6" t="n"/>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>排序信号</t>
+          <t>账号防刷</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>真实热度</t>
+          <t>机器注册防护</t>
         </is>
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>播放/完播/收藏/复制率</t>
+          <t>验证码/设备/IP/行为风控</t>
         </is>
       </c>
       <c r="F98" s="3" t="inlineStr">
         <is>
-          <t>当前互动计数真实，但推荐排序还未引入完整行为信号</t>
+          <t>当前本地登录未做注册防刷；后续优先接公司画布登录，若自建注册则必须补风控</t>
         </is>
       </c>
       <c r="G98" s="5" t="inlineStr">
@@ -4809,14 +4797,14 @@
           <t>待开发</t>
         </is>
       </c>
-      <c r="H98" s="11" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="H98" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>V2.0 增强能力</t>
+          <t>V1.1 账号生产化</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
@@ -4828,24 +4816,20 @@
     <row r="99">
       <c r="A99" s="6" t="n"/>
       <c r="B99" s="7" t="n"/>
-      <c r="C99" s="2" t="inlineStr">
-        <is>
-          <t>专题榜单</t>
-        </is>
-      </c>
+      <c r="C99" s="7" t="n"/>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>榜单/活动/专题</t>
+          <t>登录限流</t>
         </is>
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>operation config</t>
+          <t>失败次数/IP/账号锁定</t>
         </is>
       </c>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>运营层专题、榜单、活动配置待社区后台运营模块支持</t>
+          <t>登录接口上线前需限制暴力破解和撞库；当前本地登录只用于开发演示</t>
         </is>
       </c>
       <c r="G99" s="5" t="inlineStr">
@@ -4853,19 +4837,19 @@
           <t>待开发</t>
         </is>
       </c>
-      <c r="H99" s="11" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="H99" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t>V2.0 增强能力</t>
+          <t>V1.1 账号生产化</t>
         </is>
       </c>
       <c r="J99" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-21</t>
         </is>
       </c>
     </row>
@@ -4873,27 +4857,27 @@
       <c r="A100" s="6" t="n"/>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>工程与上线</t>
+          <t>推荐与运营</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>前端主线</t>
+          <t>首页分发</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>Next.js 工程</t>
+          <t>首页聚合</t>
         </is>
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>apps/web</t>
+          <t>/api/feed/home</t>
         </is>
       </c>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>正式前端主线已切到 Next.js + React + TypeScript，旧 Vite 原型已归档</t>
+          <t>首页和精选可从数据库读取内容，PGC 冷启动可演示</t>
         </is>
       </c>
       <c r="G100" s="4" t="inlineStr">
@@ -4908,7 +4892,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>V1.0 工程收口</t>
+          <t>V1.0 本地闭环</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -4922,42 +4906,42 @@
       <c r="B101" s="6" t="n"/>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>后端主线</t>
+          <t>精选运营</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>Spring Boot 工程</t>
+          <t>运营精选</t>
         </is>
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>apps/server</t>
+          <t>featured/hot</t>
         </is>
       </c>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>正式后端主线使用 Spring Boot，承接社区读写 API</t>
-        </is>
-      </c>
-      <c r="G101" s="4" t="inlineStr">
-        <is>
-          <t>已完成</t>
-        </is>
-      </c>
-      <c r="H101" s="5" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>当前精选仍以业务查询和简单排序为主；后续由 /admin/feed-ops/featured 接管人工精选与排序</t>
+        </is>
+      </c>
+      <c r="G101" s="9" t="inlineStr">
+        <is>
+          <t>开发中</t>
+        </is>
+      </c>
+      <c r="H101" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="I101" s="2" t="inlineStr">
         <is>
-          <t>V1.0 工程收口</t>
+          <t>V1.2 后台系统</t>
         </is>
       </c>
       <c r="J101" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -4966,37 +4950,37 @@
       <c r="B102" s="6" t="n"/>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>本地基础设施</t>
+          <t>搜索能力</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Docker Compose</t>
+          <t>搜索引擎</t>
         </is>
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>PostgreSQL 5432 / Redis 6379</t>
+          <t>keyword/index</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>本地数据库和缓存已可支撑全链路联调</t>
-        </is>
-      </c>
-      <c r="G102" s="4" t="inlineStr">
-        <is>
-          <t>已完成</t>
-        </is>
-      </c>
-      <c r="H102" s="5" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>尚未接搜索引擎和索引更新任务，内容规模上来后再做</t>
+        </is>
+      </c>
+      <c r="G102" s="5" t="inlineStr">
+        <is>
+          <t>待开发</t>
+        </is>
+      </c>
+      <c r="H102" s="11" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>V1.0 本地闭环</t>
+          <t>V2.0 增强能力</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
@@ -5010,130 +4994,134 @@
       <c r="B103" s="6" t="n"/>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>数据库迁移</t>
+          <t>排序信号</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>Flyway</t>
+          <t>真实热度</t>
         </is>
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>V1-V9</t>
+          <t>播放/完播/收藏/复制率</t>
         </is>
       </c>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>Flyway 已持续扩展，账号、内容、发布、互动、画布占位、讨论、提示词、后台治理与运营配置迁移脚本已落地</t>
-        </is>
-      </c>
-      <c r="G103" s="4" t="inlineStr">
-        <is>
-          <t>已完成</t>
-        </is>
-      </c>
-      <c r="H103" s="5" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>当前互动计数真实，但推荐排序还未引入完整行为信号</t>
+        </is>
+      </c>
+      <c r="G103" s="5" t="inlineStr">
+        <is>
+          <t>待开发</t>
+        </is>
+      </c>
+      <c r="H103" s="11" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>V1.1 工程化</t>
+          <t>V2.0 增强能力</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-04-21</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="6" t="n"/>
-      <c r="B104" s="6" t="n"/>
+      <c r="B104" s="7" t="n"/>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>链路追踪</t>
+          <t>专题榜单</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>requestId + traceId</t>
+          <t>榜单/活动/专题</t>
         </is>
       </c>
       <c r="E104" s="3" t="inlineStr">
         <is>
-          <t>X-Request-Id / X-Trace-Id</t>
+          <t>operation config</t>
         </is>
       </c>
       <c r="F104" s="3" t="inlineStr">
         <is>
-          <t>本地与云测试已补 requestId + traceId + userId 日志字段，便于单请求排障；异步/Worker 全链路透传待补</t>
-        </is>
-      </c>
-      <c r="G104" s="4" t="inlineStr">
-        <is>
-          <t>开发中</t>
-        </is>
-      </c>
-      <c r="H104" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>运营层专题、榜单、活动配置待社区后台运营模块支持</t>
+        </is>
+      </c>
+      <c r="G104" s="5" t="inlineStr">
+        <is>
+          <t>待开发</t>
+        </is>
+      </c>
+      <c r="H104" s="11" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>V1.1 运维化</t>
+          <t>V2.0 增强能力</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-04-27</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="6" t="n"/>
-      <c r="B105" s="6" t="n"/>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>工程与上线</t>
+        </is>
+      </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>日志体系</t>
+          <t>前端主线</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>访问/应用/错误日志</t>
+          <t>Next.js 工程</t>
         </is>
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>固定日志路径</t>
+          <t>apps/web</t>
         </is>
       </c>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>本地与云测试已具备基础日志落地和统一字段；线上采集、查询平台与告警规则待补</t>
-        </is>
-      </c>
-      <c r="G105" s="8" t="inlineStr">
-        <is>
-          <t>开发中</t>
-        </is>
-      </c>
-      <c r="H105" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>正式前端主线已切到 Next.js + React + TypeScript，旧 Vite 原型已归档</t>
+        </is>
+      </c>
+      <c r="G105" s="4" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="H105" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="I105" s="2" t="inlineStr">
         <is>
-          <t>V1.1 运维化</t>
+          <t>V1.0 工程收口</t>
         </is>
       </c>
       <c r="J105" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-04-21</t>
         </is>
       </c>
     </row>
@@ -5142,27 +5130,27 @@
       <c r="B106" s="6" t="n"/>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>线上监控</t>
+          <t>后端主线</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>指标与告警</t>
+          <t>Spring Boot 工程</t>
         </is>
       </c>
       <c r="E106" s="3" t="inlineStr">
         <is>
-          <t>QPS/错误率/延迟/队列积压</t>
+          <t>apps/server</t>
         </is>
       </c>
       <c r="F106" s="3" t="inlineStr">
         <is>
-          <t>云测试环境已跑通基础服务；监控告警、队列堆积、存储/CDN 异常监控仍待建设</t>
-        </is>
-      </c>
-      <c r="G106" s="5" t="inlineStr">
-        <is>
-          <t>待开发</t>
+          <t>正式后端主线使用 Spring Boot，承接社区读写 API</t>
+        </is>
+      </c>
+      <c r="G106" s="4" t="inlineStr">
+        <is>
+          <t>已完成</t>
         </is>
       </c>
       <c r="H106" s="5" t="inlineStr">
@@ -5172,12 +5160,12 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>V1.1 运维化</t>
+          <t>V1.0 工程收口</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-04-21</t>
         </is>
       </c>
     </row>
@@ -5186,42 +5174,42 @@
       <c r="B107" s="6" t="n"/>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>排障面板</t>
+          <t>本地基础设施</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
         <is>
-          <t>业务链路追踪</t>
+          <t>Docker Compose</t>
         </is>
       </c>
       <c r="E107" s="3" t="inlineStr">
         <is>
-          <t>发布/上传/审核/画布复制</t>
+          <t>PostgreSQL 5432 / Redis 6379</t>
         </is>
       </c>
       <c r="F107" s="3" t="inlineStr">
         <is>
-          <t>当前主要靠 requestId / traceId + 日志排查；按业务 ID 查询链路状态的排障面板待建设</t>
-        </is>
-      </c>
-      <c r="G107" s="5" t="inlineStr">
-        <is>
-          <t>待开发</t>
-        </is>
-      </c>
-      <c r="H107" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>本地数据库和缓存已可支撑全链路联调</t>
+        </is>
+      </c>
+      <c r="G107" s="4" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="H107" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>V1.1 运维化</t>
+          <t>V1.0 本地闭环</t>
         </is>
       </c>
       <c r="J107" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-04-21</t>
         </is>
       </c>
     </row>
@@ -5230,84 +5218,348 @@
       <c r="B108" s="6" t="n"/>
       <c r="C108" s="2" t="inlineStr">
         <is>
+          <t>数据库迁移</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>Flyway</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>V1-V9</t>
+        </is>
+      </c>
+      <c r="F108" s="3" t="inlineStr">
+        <is>
+          <t>Flyway 已持续扩展到 V1-V24；账号、内容、发布、互动、讨论、提示词、后台治理、运营配置等迁移脚本已落地</t>
+        </is>
+      </c>
+      <c r="G108" s="4" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="H108" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>V1.1 工程化</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="6" t="n"/>
+      <c r="B109" s="6" t="n"/>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>链路追踪</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>requestId + traceId</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>X-Request-Id / X-Trace-Id</t>
+        </is>
+      </c>
+      <c r="F109" s="3" t="inlineStr">
+        <is>
+          <t>本地与云测试已补 requestId + traceId + userId 日志字段，后台操作日志也可回看 requestId / traceId；异步/Worker 全链路透传待补</t>
+        </is>
+      </c>
+      <c r="G109" s="4" t="inlineStr">
+        <is>
+          <t>开发中</t>
+        </is>
+      </c>
+      <c r="H109" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
+          <t>V1.1 运维化</t>
+        </is>
+      </c>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="6" t="n"/>
+      <c r="B110" s="6" t="n"/>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>日志体系</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>访问/应用/错误日志</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>固定日志路径</t>
+        </is>
+      </c>
+      <c r="F110" s="3" t="inlineStr">
+        <is>
+          <t>本地与云测试已具备访问/应用/错误日志与 media_proxy_* 结构化日志；线上采集、查询平台与告警规则待补</t>
+        </is>
+      </c>
+      <c r="G110" s="8" t="inlineStr">
+        <is>
+          <t>开发中</t>
+        </is>
+      </c>
+      <c r="H110" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr">
+        <is>
+          <t>V1.1 运维化</t>
+        </is>
+      </c>
+      <c r="J110" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="6" t="n"/>
+      <c r="B111" s="6" t="n"/>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>线上监控</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>指标与告警</t>
+        </is>
+      </c>
+      <c r="E111" s="3" t="inlineStr">
+        <is>
+          <t>QPS/错误率/延迟/队列积压</t>
+        </is>
+      </c>
+      <c r="F111" s="3" t="inlineStr">
+        <is>
+          <t>云测试环境已跑通基础服务；监控告警、队列堆积、存储/CDN 异常监控仍待建设</t>
+        </is>
+      </c>
+      <c r="G111" s="5" t="inlineStr">
+        <is>
+          <t>待开发</t>
+        </is>
+      </c>
+      <c r="H111" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
+          <t>V1.1 运维化</t>
+        </is>
+      </c>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="6" t="n"/>
+      <c r="B112" s="6" t="n"/>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>排障面板</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>业务链路追踪</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>发布/上传/审核/画布复制</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>当前主要靠 requestId / traceId + 日志排查；按业务 ID 查询链路状态的排障面板待建设</t>
+        </is>
+      </c>
+      <c r="G112" s="5" t="inlineStr">
+        <is>
+          <t>待开发</t>
+        </is>
+      </c>
+      <c r="H112" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>V1.1 运维化</t>
+        </is>
+      </c>
+      <c r="J112" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="6" t="n"/>
+      <c r="B113" s="6" t="n"/>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
           <t>线上环境</t>
         </is>
       </c>
-      <c r="D108" s="3" t="inlineStr">
+      <c r="D113" s="3" t="inlineStr">
         <is>
           <t>部署与域名</t>
         </is>
       </c>
-      <c r="E108" s="3" t="inlineStr">
+      <c r="E113" s="3" t="inlineStr">
         <is>
           <t>HTTPS/Nginx/CDN/CI</t>
         </is>
       </c>
-      <c r="F108" s="3" t="inlineStr">
-        <is>
-          <t>云测试已完成 ECS + PostgreSQL(RDS) + Redis + OSS 联通并可公网试跑；HTTPS、CDN、CI/CD 与正式域名待补</t>
-        </is>
-      </c>
-      <c r="G108" s="5" t="inlineStr">
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>云测试已完成社区前台公网入口 8.141.20.130、后台入口 :3206、ECS + PostgreSQL(RDS) + Redis + 私有 OSS 联通，并已建立 release/rollback 脚本；HTTPS、CDN、正式域名与标准 CI/CD 待补</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr">
         <is>
           <t>开发中</t>
         </is>
       </c>
-      <c r="H108" s="5" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="I108" s="2" t="inlineStr">
+      <c r="H113" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I113" s="2" t="inlineStr">
         <is>
           <t>V1.1 云化改造</t>
         </is>
       </c>
-      <c r="J108" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="7" t="n"/>
-      <c r="B109" s="7" t="n"/>
-      <c r="C109" s="2" t="inlineStr">
+      <c r="J113" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="6" t="n"/>
+      <c r="B114" s="6" t="n"/>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>测试环境发布</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>release 账本与回滚</t>
+        </is>
+      </c>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>deploy/rollback/list releases</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="inlineStr">
+        <is>
+          <t>社区前台、共享后端、管理后台均已建立测试环境发布台账、当前版本查询、稳定基线与回滚脚本；标准 CI/CD 仍待补</t>
+        </is>
+      </c>
+      <c r="G114" s="5" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="H114" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I114" s="2" t="inlineStr">
+        <is>
+          <t>V1.1 运维化</t>
+        </is>
+      </c>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="7" t="n"/>
+      <c r="B115" s="7" t="n"/>
+      <c r="C115" s="2" t="inlineStr">
         <is>
           <t>备份恢复</t>
         </is>
       </c>
-      <c r="D109" s="3" t="inlineStr">
+      <c r="D115" s="3" t="inlineStr">
         <is>
           <t>数据备份</t>
         </is>
       </c>
-      <c r="E109" s="3" t="inlineStr">
+      <c r="E115" s="3" t="inlineStr">
         <is>
           <t>PostgreSQL/Object Storage</t>
         </is>
       </c>
-      <c r="F109" s="3" t="inlineStr">
+      <c r="F115" s="3" t="inlineStr">
         <is>
           <t>上线前需要数据库备份、对象存储生命周期和恢复演练</t>
         </is>
       </c>
-      <c r="G109" s="5" t="inlineStr">
+      <c r="G115" s="5" t="inlineStr">
         <is>
           <t>待开发</t>
         </is>
       </c>
-      <c r="H109" s="8" t="inlineStr">
+      <c r="H115" s="8" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="I109" s="2" t="inlineStr">
+      <c r="I115" s="2" t="inlineStr">
         <is>
           <t>V1.1 运维化</t>
         </is>
       </c>
-      <c r="J109" s="2" t="inlineStr">
+      <c r="J115" s="2" t="inlineStr">
         <is>
           <t>2026-04-21</t>
         </is>
@@ -5364,7 +5616,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="90" customWidth="1" min="2" max="2"/>
@@ -5378,7 +5630,7 @@
       </c>
       <c r="B1" s="13" t="inlineStr">
         <is>
-          <t>PGC 冷启动阶段，前台社区主线已基本跑通，正在进入云测试与后台一期并行阶段</t>
+          <t>PGC 冷启动阶段，社区前台主链路、云测试链路与后台一期已跑通，当前进入生产化补齐阶段</t>
         </is>
       </c>
     </row>
@@ -5390,7 +5642,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>当前重点是继续收口前台发布/评论/详情体验，推进后台一期（账号、审核、举报、运营配置），并补 OSS/CDN、媒体 Worker、公司登录与监控能力</t>
+          <t>当前重点是继续收口媒体云化 T6 后续事项，推进后台二期治理，并补公网 OSS/CDN、预签名直传、独立 Worker、公司登录、监控告警与 CI/CD</t>
         </is>
       </c>
     </row>
@@ -5402,7 +5654,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>状态按当前代码、云测试现状与进度文档综合判断；区分社区前台、社区后台与共用能力，不把计划态能力写成已完成</t>
+          <t>状态已同步到 2026-05-24 的前后台代码、云测试发布台账、主进度文档与社区后台共享文档；已完成只写真实可验收能力</t>
         </is>
       </c>
     </row>
@@ -5414,7 +5666,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>首页分发 -&gt; 精选/详情 -&gt; 作者主页 -&gt; 发布 -&gt; 互动 -&gt; 画布入口 -&gt; 后台治理</t>
+          <t>首页分发 -&gt; 精选/详情 -&gt; 发布 -&gt; 互动 -&gt; /me 与作者主页 -&gt; 后台审核/举报/运营 -&gt; 云媒体链路</t>
         </is>
       </c>
     </row>
@@ -5426,7 +5678,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>距离完整上线仍缺 HTTPS/CDN/CI-CD、媒体转码与预览生成、公司登录、后台剩余治理、监控告警与更完整内容安全</t>
+          <t>距离完整上线仍缺 HTTPS/正式域名/CDN、公网或受控 OSS 访问、预签名直传与分片上传、独立媒体 Worker/队列、公司统一登录、监控告警与标准 CI/CD</t>
         </is>
       </c>
     </row>

</xml_diff>